<commit_message>
feat: update squish tracker with updated BOM state, parts list, and CAD features
</commit_message>
<xml_diff>
--- a/tracker/Parts List.xlsx
+++ b/tracker/Parts List.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="56">
   <si>
     <t>Categrory</t>
   </si>
@@ -100,9 +100,6 @@
     <t>STM32 Blackpill MCU</t>
   </si>
   <si>
-    <t>STM32F411 BlackPill Dev</t>
-  </si>
-  <si>
     <t>H-Bridge Driver</t>
   </si>
   <si>
@@ -115,7 +112,10 @@
     <t>ADC</t>
   </si>
   <si>
-    <t>NAU7802</t>
+    <t>NAU7802 - 4538</t>
+  </si>
+  <si>
+    <t>ADC Cable</t>
   </si>
   <si>
     <t>Logic Level Shifter</t>
@@ -127,22 +127,22 @@
     <t>Mechanical</t>
   </si>
   <si>
-    <t xml:space="preserve"> Inner Rails</t>
-  </si>
-  <si>
-    <t>Online Metals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nonperforated </t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.3lbs </t>
+    <t>Main Rail</t>
+  </si>
+  <si>
+    <t>Inner Rails</t>
+  </si>
+  <si>
+    <t>McMaster</t>
+  </si>
+  <si>
+    <t>updated for larger inside space</t>
   </si>
   <si>
     <t>Outer Rails</t>
   </si>
   <si>
-    <t xml:space="preserve">0.47lbs </t>
+    <t>- if too much wiggle room due to tolerances, friction wear pads</t>
   </si>
   <si>
     <t xml:space="preserve">M4 Screws </t>
@@ -157,10 +157,28 @@
     <t xml:space="preserve">Amazon </t>
   </si>
   <si>
-    <t>1.57''x0.31''</t>
+    <t>9.6mm x 50 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">length 2 inches </t>
   </si>
   <si>
     <t xml:space="preserve">Load Cell Spacers </t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D Print </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Framing </t>
+  </si>
+  <si>
+    <t>T-slot frames</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-slot end caps </t>
+  </si>
+  <si>
+    <t>Mounting Plate</t>
   </si>
 </sst>
 </file>
@@ -171,7 +189,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -194,6 +212,10 @@
       <color rgb="FF0000FF"/>
     </font>
     <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -202,12 +224,18 @@
       <color rgb="FF0000FF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB6D7A8"/>
+        <bgColor rgb="FFB6D7A8"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -228,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -254,19 +282,31 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -566,16 +606,16 @@
     </row>
     <row r="4">
       <c r="A4" s="8"/>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="11">
         <v>4.0</v>
       </c>
       <c r="F4" s="5" t="s">
@@ -602,16 +642,16 @@
     </row>
     <row r="6">
       <c r="A6" s="8"/>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="11">
         <v>10.0</v>
       </c>
     </row>
@@ -622,16 +662,16 @@
       <c r="A8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="12">
         <v>10.0</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -643,7 +683,7 @@
       <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="10"/>
+      <c r="C9" s="13"/>
       <c r="E9" s="7" t="s">
         <v>18</v>
       </c>
@@ -653,26 +693,26 @@
     </row>
     <row r="10">
       <c r="A10" s="8"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="C10" s="10">
+        <v>4877.0</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="11">
         <v>30.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8"/>
       <c r="B11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>31</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>17</v>
@@ -681,128 +721,165 @@
         <v>15.0</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8"/>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="11">
         <v>6.0</v>
       </c>
       <c r="F12" s="5"/>
     </row>
     <row r="13">
       <c r="A13" s="8"/>
-      <c r="B13" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="13">
-        <v>7.0</v>
-      </c>
+      <c r="B13" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="10">
+        <v>4397.0</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="F13" s="5"/>
     </row>
     <row r="14">
       <c r="A14" s="8"/>
+      <c r="B14" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="16">
+        <v>7.0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="8"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="9">
-        <v>7.36</v>
-      </c>
-      <c r="F16" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="E17" s="17">
+        <v>11.66</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8"/>
-      <c r="C17" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="9">
-        <v>7.93</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8"/>
-      <c r="C18" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>45</v>
+      <c r="C18" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="17">
+        <v>21.48</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8"/>
-      <c r="C19" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" s="9">
-        <v>9.99</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>48</v>
+      <c r="C19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8"/>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="17">
+        <v>10.99</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8"/>
+      <c r="C21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8"/>
+      <c r="B22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8"/>
+      <c r="C23" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8"/>
+      <c r="C24" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8"/>
@@ -3737,6 +3814,9 @@
     </row>
     <row r="1002">
       <c r="A1002" s="8"/>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3750,10 +3830,11 @@
     <hyperlink r:id="rId8" ref="C11"/>
     <hyperlink r:id="rId9" ref="C12"/>
     <hyperlink r:id="rId10" ref="C13"/>
-    <hyperlink r:id="rId11" ref="C16"/>
+    <hyperlink r:id="rId11" ref="C14"/>
     <hyperlink r:id="rId12" ref="C17"/>
-    <hyperlink r:id="rId13" ref="C19"/>
+    <hyperlink r:id="rId13" ref="C18"/>
+    <hyperlink r:id="rId14" ref="C20"/>
   </hyperlinks>
-  <drawing r:id="rId14"/>
+  <drawing r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>